<commit_message>
Added New tc -58 of defect page,& updated execute tab tc-41 to tc-80
</commit_message>
<xml_diff>
--- a/testData/executeTestCaseTabTestData/executeTestCaseTab_testData.xlsx
+++ b/testData/executeTestCaseTabTestData/executeTestCaseTab_testData.xlsx
@@ -1,76 +1,87 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29728"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29825"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0A4E9934-3AD6-4655-8A09-F73BCB19CE2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B5608523-139B-4D58-86F1-B65CD3F1C470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="58" activeTab="58" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="69" activeTab="69" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tc001" sheetId="1" r:id="rId1"/>
-    <sheet name="tc014" sheetId="27" r:id="rId2"/>
-    <sheet name="tc042" sheetId="20" r:id="rId3"/>
-    <sheet name="tc019" sheetId="28" r:id="rId4"/>
-    <sheet name="tc029" sheetId="38" r:id="rId5"/>
-    <sheet name="tc028" sheetId="29" r:id="rId6"/>
-    <sheet name="tc002" sheetId="4" r:id="rId7"/>
-    <sheet name="tc003" sheetId="2" r:id="rId8"/>
-    <sheet name="tc004" sheetId="3" r:id="rId9"/>
-    <sheet name="tc006" sheetId="5" r:id="rId10"/>
-    <sheet name="tc044" sheetId="37" r:id="rId11"/>
-    <sheet name="tc032" sheetId="42" r:id="rId12"/>
-    <sheet name="tc026" sheetId="43" r:id="rId13"/>
-    <sheet name="tc007" sheetId="8" r:id="rId14"/>
-    <sheet name="tc025" sheetId="45" r:id="rId15"/>
-    <sheet name="tc009" sheetId="13" r:id="rId16"/>
-    <sheet name="tc011" sheetId="6" r:id="rId17"/>
-    <sheet name="tc013" sheetId="7" r:id="rId18"/>
-    <sheet name="tc015" sheetId="9" r:id="rId19"/>
-    <sheet name="tc016" sheetId="11" r:id="rId20"/>
-    <sheet name="tc018" sheetId="18" r:id="rId21"/>
-    <sheet name="tc017" sheetId="46" r:id="rId22"/>
-    <sheet name="tc043" sheetId="26" r:id="rId23"/>
-    <sheet name="tc037" sheetId="34" r:id="rId24"/>
-    <sheet name="tc021" sheetId="14" r:id="rId25"/>
-    <sheet name="tc022" sheetId="30" r:id="rId26"/>
-    <sheet name="tc024" sheetId="31" r:id="rId27"/>
-    <sheet name="tc031" sheetId="32" r:id="rId28"/>
-    <sheet name="tc023" sheetId="10" r:id="rId29"/>
-    <sheet name="tc034" sheetId="15" r:id="rId30"/>
-    <sheet name="tc036" sheetId="12" r:id="rId31"/>
-    <sheet name="tc038" sheetId="17" r:id="rId32"/>
-    <sheet name="tc039" sheetId="16" r:id="rId33"/>
-    <sheet name="tc040" sheetId="19" r:id="rId34"/>
-    <sheet name="tc045" sheetId="25" r:id="rId35"/>
-    <sheet name="tc046" sheetId="33" r:id="rId36"/>
-    <sheet name="tc047" sheetId="21" r:id="rId37"/>
-    <sheet name="tc048" sheetId="22" r:id="rId38"/>
-    <sheet name="tc049" sheetId="24" r:id="rId39"/>
-    <sheet name="tc050" sheetId="36" r:id="rId40"/>
-    <sheet name="tc020" sheetId="39" r:id="rId41"/>
-    <sheet name="tc010" sheetId="44" r:id="rId42"/>
-    <sheet name="tc041" sheetId="41" r:id="rId43"/>
-    <sheet name="tc059" sheetId="48" r:id="rId44"/>
-    <sheet name="tc060" sheetId="49" r:id="rId45"/>
-    <sheet name="tc061" sheetId="51" r:id="rId46"/>
-    <sheet name="tc062" sheetId="52" r:id="rId47"/>
-    <sheet name="tc063" sheetId="47" r:id="rId48"/>
-    <sheet name="tc064" sheetId="50" r:id="rId49"/>
-    <sheet name="tc065" sheetId="53" r:id="rId50"/>
-    <sheet name="tc066" sheetId="54" r:id="rId51"/>
-    <sheet name="tc071" sheetId="55" r:id="rId52"/>
-    <sheet name="tc072" sheetId="60" r:id="rId53"/>
-    <sheet name="tc073" sheetId="61" r:id="rId54"/>
-    <sheet name="tc074" sheetId="62" r:id="rId55"/>
-    <sheet name="tc075" sheetId="63" r:id="rId56"/>
-    <sheet name="tc076" sheetId="64" r:id="rId57"/>
-    <sheet name="tc077" sheetId="65" r:id="rId58"/>
-    <sheet name="tc078" sheetId="66" r:id="rId59"/>
-    <sheet name="tc067" sheetId="56" r:id="rId60"/>
-    <sheet name="tc068" sheetId="57" r:id="rId61"/>
-    <sheet name="tc069" sheetId="58" r:id="rId62"/>
-    <sheet name="tc070" sheetId="59" r:id="rId63"/>
+    <sheet name="tc008" sheetId="68" r:id="rId2"/>
+    <sheet name="tc014" sheetId="27" r:id="rId3"/>
+    <sheet name="tc042" sheetId="20" r:id="rId4"/>
+    <sheet name="tc019" sheetId="28" r:id="rId5"/>
+    <sheet name="tc029" sheetId="38" r:id="rId6"/>
+    <sheet name="tc028" sheetId="29" r:id="rId7"/>
+    <sheet name="tc002" sheetId="4" r:id="rId8"/>
+    <sheet name="tc003" sheetId="2" r:id="rId9"/>
+    <sheet name="tc004" sheetId="3" r:id="rId10"/>
+    <sheet name="tc012" sheetId="69" r:id="rId11"/>
+    <sheet name="tc006" sheetId="5" r:id="rId12"/>
+    <sheet name="tc044" sheetId="37" r:id="rId13"/>
+    <sheet name="tc055" sheetId="74" r:id="rId14"/>
+    <sheet name="tc056" sheetId="75" r:id="rId15"/>
+    <sheet name="tc057" sheetId="76" r:id="rId16"/>
+    <sheet name="tc032" sheetId="42" r:id="rId17"/>
+    <sheet name="tc026" sheetId="43" r:id="rId18"/>
+    <sheet name="tc007" sheetId="8" r:id="rId19"/>
+    <sheet name="tc025" sheetId="45" r:id="rId20"/>
+    <sheet name="tc009" sheetId="13" r:id="rId21"/>
+    <sheet name="tc011" sheetId="6" r:id="rId22"/>
+    <sheet name="tc013" sheetId="7" r:id="rId23"/>
+    <sheet name="tc015" sheetId="9" r:id="rId24"/>
+    <sheet name="tc016" sheetId="11" r:id="rId25"/>
+    <sheet name="tc018" sheetId="18" r:id="rId26"/>
+    <sheet name="tc017" sheetId="46" r:id="rId27"/>
+    <sheet name="tc043" sheetId="26" r:id="rId28"/>
+    <sheet name="tc037" sheetId="34" r:id="rId29"/>
+    <sheet name="tc021" sheetId="14" r:id="rId30"/>
+    <sheet name="tc022" sheetId="30" r:id="rId31"/>
+    <sheet name="tc024" sheetId="31" r:id="rId32"/>
+    <sheet name="tc031" sheetId="32" r:id="rId33"/>
+    <sheet name="tc051" sheetId="70" r:id="rId34"/>
+    <sheet name="tc023" sheetId="10" r:id="rId35"/>
+    <sheet name="tc053" sheetId="72" r:id="rId36"/>
+    <sheet name="tc054" sheetId="73" r:id="rId37"/>
+    <sheet name="tc034" sheetId="15" r:id="rId38"/>
+    <sheet name="tc036" sheetId="12" r:id="rId39"/>
+    <sheet name="tc038" sheetId="17" r:id="rId40"/>
+    <sheet name="tc039" sheetId="16" r:id="rId41"/>
+    <sheet name="tc040" sheetId="19" r:id="rId42"/>
+    <sheet name="tc045" sheetId="25" r:id="rId43"/>
+    <sheet name="tc046" sheetId="33" r:id="rId44"/>
+    <sheet name="tc047" sheetId="21" r:id="rId45"/>
+    <sheet name="tc048" sheetId="22" r:id="rId46"/>
+    <sheet name="tc049" sheetId="24" r:id="rId47"/>
+    <sheet name="tc050" sheetId="36" r:id="rId48"/>
+    <sheet name="tc052" sheetId="71" r:id="rId49"/>
+    <sheet name="tc020" sheetId="39" r:id="rId50"/>
+    <sheet name="tc010" sheetId="44" r:id="rId51"/>
+    <sheet name="tc041" sheetId="41" r:id="rId52"/>
+    <sheet name="tc059" sheetId="48" r:id="rId53"/>
+    <sheet name="tc060" sheetId="49" r:id="rId54"/>
+    <sheet name="tc061" sheetId="51" r:id="rId55"/>
+    <sheet name="tc062" sheetId="52" r:id="rId56"/>
+    <sheet name="tc063" sheetId="47" r:id="rId57"/>
+    <sheet name="tc064" sheetId="50" r:id="rId58"/>
+    <sheet name="tc065" sheetId="53" r:id="rId59"/>
+    <sheet name="tc066" sheetId="54" r:id="rId60"/>
+    <sheet name="tc071" sheetId="55" r:id="rId61"/>
+    <sheet name="tc072" sheetId="60" r:id="rId62"/>
+    <sheet name="tc073" sheetId="61" r:id="rId63"/>
+    <sheet name="tc074" sheetId="62" r:id="rId64"/>
+    <sheet name="tc075" sheetId="63" r:id="rId65"/>
+    <sheet name="tc076" sheetId="64" r:id="rId66"/>
+    <sheet name="tc077" sheetId="65" r:id="rId67"/>
+    <sheet name="tc078" sheetId="66" r:id="rId68"/>
+    <sheet name="tc079" sheetId="67" r:id="rId69"/>
+    <sheet name="tc080" sheetId="77" r:id="rId70"/>
+    <sheet name="tc067" sheetId="56" r:id="rId71"/>
+    <sheet name="tc068" sheetId="57" r:id="rId72"/>
+    <sheet name="tc069" sheetId="58" r:id="rId73"/>
+    <sheet name="tc070" sheetId="59" r:id="rId74"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -93,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="130">
   <si>
     <t>projectName</t>
   </si>
@@ -353,6 +364,9 @@
     <t>TC-427</t>
   </si>
   <si>
+    <t>tc</t>
+  </si>
+  <si>
     <t>defid</t>
   </si>
   <si>
@@ -381,9 +395,6 @@
   </si>
   <si>
     <t>rq</t>
-  </si>
-  <si>
-    <t>tc</t>
   </si>
   <si>
     <t>TestCycle TR Notification 12-01-2026</t>
@@ -959,6 +970,88 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CF5A029-64A1-403A-837B-C32E1E2D6417}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="32.140625" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82C5533E-46B7-404F-B141-BA8D149ED6E2}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67D36684-4EDA-4FF0-85DD-1EA9CD94F353}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1009,7 +1102,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE4B7E90-5E45-412C-A63B-679C413C3D5C}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1047,7 +1140,103 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51CCB92C-EDEC-48CF-89CB-C9462950544E}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA114ADC-2537-4EF7-8F50-85932949F6E5}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{042B7EE0-F346-47F6-9722-542962CA49F2}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988F8CE0-D2B6-4607-9F68-E84B3BB17A0A}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1085,7 +1274,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DF7D1D6-42F9-4EC1-BFA9-B2A7D34CCAC2}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1123,7 +1312,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D4354BF-6006-4215-AA04-8EA9BBA3CDF1}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultColWidth="27.140625" defaultRowHeight="15"/>
@@ -1167,7 +1356,33 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82C2809E-16FE-43EA-BC05-80D276E43A65}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F957C3CC-73B2-4386-9703-3136A7AE8A62}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="14.85546875" defaultRowHeight="15"/>
@@ -1205,7 +1420,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33EC2AFD-EEAB-4A46-AE51-DB66407041B8}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1242,7 +1457,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A085FA3-2BB3-4D74-980D-561D1731E50F}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1292,7 +1507,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{529C7ADA-95D5-4FFD-8278-7A1FFD92FC6F}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1359,7 +1574,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC0268C7-979F-44DB-BB29-34F2B8A2CC61}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1421,49 +1636,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAE3D50E-9B7C-4048-BF74-2691F8F3F3B0}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="27" customWidth="1"/>
-    <col min="2" max="2" width="19.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0EDD7F5-B476-4FD1-BEDA-E531A4CC894D}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1519,7 +1692,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53291E11-0F73-43B9-A291-8813C6E50618}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1575,7 +1748,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8956054-5465-4015-AEAB-67BB9851B24F}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultColWidth="18.28515625" defaultRowHeight="15"/>
@@ -1619,7 +1792,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C5EDEDE-C2C9-4A01-9CD5-CB8C86EBBE08}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1662,7 +1835,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20AD7FB8-5DA1-4488-9DE3-A42870B02C3F}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1700,7 +1873,49 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAE3D50E-9B7C-4048-BF74-2691F8F3F3B0}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90FECA65-C9A0-48C7-B3DC-F9FDF05C4662}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1744,7 +1959,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB0829FE-96F7-43C0-8C41-619F29B6B47C}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultColWidth="14" defaultRowHeight="15"/>
@@ -1794,107 +2009,145 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60A730C5-C7A1-4920-B9BC-7469CD655A62}">
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultColWidth="17.140625" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F1" t="s">
+        <v>63</v>
+      </c>
+      <c r="G1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="F2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C9A404D-916D-4310-B74F-6006281B7179}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="23.5703125" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C499954-818C-4267-A95A-C13609BD2025}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="17.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E1" t="s">
-        <v>63</v>
+        <v>13</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="F1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>7</v>
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="E2" t="s">
-        <v>66</v>
-      </c>
-      <c r="F2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C9A404D-916D-4310-B74F-6006281B7179}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="23.5703125" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="E2" t="s">
-        <v>66</v>
-      </c>
-      <c r="F2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>24</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1184356D-1AE6-4E98-8694-D387B6BCDC24}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1931,62 +2184,71 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{807E892B-8929-4105-B8A9-12065D70D1F4}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="12.28515625" customWidth="1"/>
-    <col min="2" max="2" width="33.42578125" customWidth="1"/>
-    <col min="6" max="6" width="28" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F2" s="10" t="s">
-        <v>20</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{602CC745-32D4-47CB-82A6-B4E20CF5EEBB}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B5AA7B5-E8E5-4566-8F96-53EECD2B45C9}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50EB1A7D-DC52-4713-ABC3-596E81595BB1}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2057,7 +2319,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDB454D5-570E-40AD-BB2C-FF13FAD6F69C}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2101,7 +2363,62 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{807E892B-8929-4105-B8A9-12065D70D1F4}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.28515625" customWidth="1"/>
+    <col min="2" max="2" width="33.42578125" customWidth="1"/>
+    <col min="6" max="6" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1ED00A0B-CD51-4A4F-8051-1ED251D3C5B6}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2151,7 +2468,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE51A2BC-36BD-4EBA-8604-26295ECE93E9}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2181,7 +2498,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B69D1B4E-F873-4DB0-B2EA-24B046130852}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2232,7 +2549,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6166FFA-72F8-495E-9A03-1D63C7A066F4}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2288,7 +2605,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{626481C8-CDB8-4E7E-84A8-4409E5CFD495}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultColWidth="24.140625" defaultRowHeight="15"/>
@@ -2338,7 +2655,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4983F34-AE5D-40C9-BB36-540F7984E580}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2400,7 +2717,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{631D63AD-491D-498E-BAC2-4C00217678C8}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2444,7 +2761,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4D278FD-C072-43D7-9D65-282A374E276D}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2506,51 +2823,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1227A506-805A-4764-8A9B-E0A3E88E40BF}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="26.42578125" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{262279DB-08EA-408F-8B51-34383F1C571D}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2620,7 +2893,113 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A5094B1-F969-40E8-B638-30CC9EEEC009}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" s="6">
+        <v>1</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1227A506-805A-4764-8A9B-E0A3E88E40BF}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultColWidth="26.42578125" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A469181C-01B9-4C34-A427-3D7B86980067}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2642,7 +3021,7 @@
         <v>53</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -2662,15 +3041,15 @@
         <v>25</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>87</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F814BA2-835C-42C7-BBDB-409A7725E7FE}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultColWidth="25.140625" defaultRowHeight="15"/>
@@ -2714,7 +3093,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3ACD041-5E11-4FA0-B069-3C5CC2C19A0C}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2739,13 +3118,13 @@
         <v>53</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G1" s="8" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -2765,21 +3144,21 @@
         <v>25</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>66</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>91</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>92</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD8F4123-7EDA-4FD6-8DA8-8DB314949234}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2794,13 +3173,13 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D1" t="s">
         <v>78</v>
@@ -2809,10 +3188,10 @@
         <v>79</v>
       </c>
       <c r="F1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G1" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -2843,7 +3222,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C530097-25F5-490E-B95D-3F7CE84A8B5A}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2859,13 +3238,13 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D1" t="s">
         <v>78</v>
@@ -2874,10 +3253,10 @@
         <v>79</v>
       </c>
       <c r="F1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G1" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="H1" t="s">
         <v>100</v>
@@ -2914,7 +3293,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9928D07B-EC4B-4FB7-A544-ACD154E60B5A}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2924,13 +3303,13 @@
         <v>101</v>
       </c>
       <c r="B1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E1" t="s">
         <v>78</v>
@@ -2939,10 +3318,10 @@
         <v>79</v>
       </c>
       <c r="G1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H1" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -2976,20 +3355,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65567DB9-F4A5-4991-BBBB-B0966631BE02}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D1" t="s">
         <v>78</v>
@@ -2998,10 +3377,10 @@
         <v>79</v>
       </c>
       <c r="F1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G1" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="H1" t="s">
         <v>100</v>
@@ -3038,7 +3417,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABC46D15-7486-489E-8CFB-3757E997A7F3}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3062,15 +3441,15 @@
         <v>105</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3493DC4-C417-4C28-8EE7-B8304F691C93}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3094,15 +3473,47 @@
         <v>105</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5737D2A7-9183-4F17-A1A0-D46634DAE493}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE4FC528-53EE-4A96-BCAB-C9D74542958B}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3139,8 +3550,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5737D2A7-9183-4F17-A1A0-D46634DAE493}">
+<file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB8F0DCE-952C-484A-B429-28D41548BB7A}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -3171,39 +3582,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB8F0DCE-952C-484A-B429-28D41548BB7A}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8840A44C-6BDB-471E-B7F3-2A372A7C4B5B}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultColWidth="19.42578125" defaultRowHeight="15"/>
@@ -3235,7 +3614,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B9B72EB-97C0-4405-94F5-046368E85D80}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3267,7 +3646,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09FCDA05-EF6F-42AB-9CB8-2EAB3573710B}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3305,7 +3684,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B038332-BB0C-4E20-A6A2-9F7526C4D248}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3343,7 +3722,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E093CE88-AC07-4898-81D8-6061F00C4D92}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3359,7 +3738,7 @@
         <v>78</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>117</v>
@@ -3387,7 +3766,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAFE400E-814A-476C-9FF3-1A384DD6A39D}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3403,7 +3782,7 @@
         <v>78</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>117</v>
@@ -3443,7 +3822,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DBB2522-C0DE-4085-ADBF-7FE9C84B6F31}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="18.140625" defaultRowHeight="15"/>
@@ -3481,7 +3860,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E1B32B0-F3F2-47B6-A128-2992201FC613}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultColWidth="19.7109375" defaultRowHeight="15"/>
@@ -3505,15 +3884,47 @@
         <v>129</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E7BB830-EB99-49CB-BF04-A0C705F8DA3E}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E32429F3-AABC-45DD-B647-116877616A3B}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3563,8 +3974,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D109D0F-DF6D-4E54-A85C-F205345D7EE8}">
+<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57E304D9-C2CF-4191-B2D5-F19B4BAEF075}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -3573,6 +3984,38 @@
         <v>107</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D109D0F-DF6D-4E54-A85C-F205345D7EE8}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>108</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -3595,7 +4038,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58DC1A5D-B5FD-4AF6-9CE0-84600C30705B}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3627,7 +4070,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AF5112D-7B38-4AF6-8BE8-212DFAB6FA1F}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3659,7 +4102,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C3DEA2D-3BC8-46BF-82C0-FA72EAFC6314}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3691,7 +4134,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84A7507B-FC99-4CF2-AE3D-BE5F23D6F22B}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultColWidth="22.85546875" defaultRowHeight="15"/>
@@ -3711,7 +4154,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{080476E3-62E4-4BCA-8888-D4B5BD88468D}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3746,48 +4189,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CF5A029-64A1-403A-837B-C32E1E2D6417}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="32.140625" customWidth="1"/>
-    <col min="2" max="2" width="19.28515625" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" customWidth="1"/>
-    <col min="4" max="4" width="14.28515625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
updated execute testcases and its locators
</commit_message>
<xml_diff>
--- a/testData/executeTestCaseTabTestData/executeTestCaseTab_testData.xlsx
+++ b/testData/executeTestCaseTabTestData/executeTestCaseTab_testData.xlsx
@@ -1,11 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29825"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B5608523-139B-4D58-86F1-B65CD3F1C470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="69" activeTab="69" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="19200" windowHeight="6800" firstSheet="32" activeTab="38"/>
   </bookViews>
   <sheets>
     <sheet name="tc001" sheetId="1" r:id="rId1"/>
@@ -39,55 +38,56 @@
     <sheet name="tc037" sheetId="34" r:id="rId29"/>
     <sheet name="tc021" sheetId="14" r:id="rId30"/>
     <sheet name="tc022" sheetId="30" r:id="rId31"/>
-    <sheet name="tc024" sheetId="31" r:id="rId32"/>
-    <sheet name="tc031" sheetId="32" r:id="rId33"/>
-    <sheet name="tc051" sheetId="70" r:id="rId34"/>
-    <sheet name="tc023" sheetId="10" r:id="rId35"/>
-    <sheet name="tc053" sheetId="72" r:id="rId36"/>
-    <sheet name="tc054" sheetId="73" r:id="rId37"/>
-    <sheet name="tc034" sheetId="15" r:id="rId38"/>
-    <sheet name="tc036" sheetId="12" r:id="rId39"/>
-    <sheet name="tc038" sheetId="17" r:id="rId40"/>
-    <sheet name="tc039" sheetId="16" r:id="rId41"/>
-    <sheet name="tc040" sheetId="19" r:id="rId42"/>
-    <sheet name="tc045" sheetId="25" r:id="rId43"/>
-    <sheet name="tc046" sheetId="33" r:id="rId44"/>
-    <sheet name="tc047" sheetId="21" r:id="rId45"/>
-    <sheet name="tc048" sheetId="22" r:id="rId46"/>
-    <sheet name="tc049" sheetId="24" r:id="rId47"/>
-    <sheet name="tc050" sheetId="36" r:id="rId48"/>
-    <sheet name="tc052" sheetId="71" r:id="rId49"/>
-    <sheet name="tc020" sheetId="39" r:id="rId50"/>
-    <sheet name="tc010" sheetId="44" r:id="rId51"/>
-    <sheet name="tc041" sheetId="41" r:id="rId52"/>
-    <sheet name="tc059" sheetId="48" r:id="rId53"/>
-    <sheet name="tc060" sheetId="49" r:id="rId54"/>
-    <sheet name="tc061" sheetId="51" r:id="rId55"/>
-    <sheet name="tc062" sheetId="52" r:id="rId56"/>
-    <sheet name="tc063" sheetId="47" r:id="rId57"/>
-    <sheet name="tc064" sheetId="50" r:id="rId58"/>
-    <sheet name="tc065" sheetId="53" r:id="rId59"/>
-    <sheet name="tc066" sheetId="54" r:id="rId60"/>
-    <sheet name="tc071" sheetId="55" r:id="rId61"/>
-    <sheet name="tc072" sheetId="60" r:id="rId62"/>
-    <sheet name="tc073" sheetId="61" r:id="rId63"/>
-    <sheet name="tc074" sheetId="62" r:id="rId64"/>
-    <sheet name="tc075" sheetId="63" r:id="rId65"/>
-    <sheet name="tc076" sheetId="64" r:id="rId66"/>
-    <sheet name="tc077" sheetId="65" r:id="rId67"/>
-    <sheet name="tc078" sheetId="66" r:id="rId68"/>
-    <sheet name="tc079" sheetId="67" r:id="rId69"/>
-    <sheet name="tc080" sheetId="77" r:id="rId70"/>
-    <sheet name="tc067" sheetId="56" r:id="rId71"/>
-    <sheet name="tc068" sheetId="57" r:id="rId72"/>
-    <sheet name="tc069" sheetId="58" r:id="rId73"/>
-    <sheet name="tc070" sheetId="59" r:id="rId74"/>
+    <sheet name="tc031" sheetId="32" r:id="rId32"/>
+    <sheet name="tc051" sheetId="70" r:id="rId33"/>
+    <sheet name="tc023" sheetId="10" r:id="rId34"/>
+    <sheet name="tc053" sheetId="72" r:id="rId35"/>
+    <sheet name="tc054" sheetId="73" r:id="rId36"/>
+    <sheet name="tc034" sheetId="15" r:id="rId37"/>
+    <sheet name="tc036" sheetId="12" r:id="rId38"/>
+    <sheet name="tc038" sheetId="17" r:id="rId39"/>
+    <sheet name="tc039" sheetId="16" r:id="rId40"/>
+    <sheet name="tc040" sheetId="19" r:id="rId41"/>
+    <sheet name="tc045" sheetId="25" r:id="rId42"/>
+    <sheet name="tc046" sheetId="33" r:id="rId43"/>
+    <sheet name="tc047" sheetId="21" r:id="rId44"/>
+    <sheet name="tc048" sheetId="22" r:id="rId45"/>
+    <sheet name="tc049" sheetId="24" r:id="rId46"/>
+    <sheet name="tc050" sheetId="36" r:id="rId47"/>
+    <sheet name="tc052" sheetId="71" r:id="rId48"/>
+    <sheet name="tc020" sheetId="39" r:id="rId49"/>
+    <sheet name="tc010" sheetId="44" r:id="rId50"/>
+    <sheet name="tc041" sheetId="41" r:id="rId51"/>
+    <sheet name="tc059" sheetId="48" r:id="rId52"/>
+    <sheet name="tc060" sheetId="49" r:id="rId53"/>
+    <sheet name="tc061" sheetId="51" r:id="rId54"/>
+    <sheet name="tc062" sheetId="52" r:id="rId55"/>
+    <sheet name="tc063" sheetId="47" r:id="rId56"/>
+    <sheet name="tc064" sheetId="50" r:id="rId57"/>
+    <sheet name="tc065" sheetId="53" r:id="rId58"/>
+    <sheet name="tc066" sheetId="54" r:id="rId59"/>
+    <sheet name="tc071" sheetId="55" r:id="rId60"/>
+    <sheet name="tc072" sheetId="60" r:id="rId61"/>
+    <sheet name="tc073" sheetId="61" r:id="rId62"/>
+    <sheet name="tc074" sheetId="62" r:id="rId63"/>
+    <sheet name="tc075" sheetId="63" r:id="rId64"/>
+    <sheet name="tc076" sheetId="64" r:id="rId65"/>
+    <sheet name="tc077" sheetId="65" r:id="rId66"/>
+    <sheet name="tc078" sheetId="66" r:id="rId67"/>
+    <sheet name="tc079" sheetId="67" r:id="rId68"/>
+    <sheet name="tc080" sheetId="77" r:id="rId69"/>
+    <sheet name="tc067" sheetId="56" r:id="rId70"/>
+    <sheet name="tc068" sheetId="57" r:id="rId71"/>
+    <sheet name="tc069" sheetId="58" r:id="rId72"/>
+    <sheet name="tc070" sheetId="59" r:id="rId73"/>
+    <sheet name="tc087" sheetId="78" r:id="rId74"/>
+    <sheet name="tc089" sheetId="79" r:id="rId75"/>
+    <sheet name="tc024" sheetId="80" r:id="rId76"/>
+    <sheet name="tc090" sheetId="81" r:id="rId77"/>
+    <sheet name="tc091" sheetId="82" r:id="rId78"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -104,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="132">
   <si>
     <t>projectName</t>
   </si>
@@ -265,6 +265,9 @@
     <t>DF-315</t>
   </si>
   <si>
+    <t>Vivek Testcycle</t>
+  </si>
+  <si>
     <t>TCClick</t>
   </si>
   <si>
@@ -322,9 +325,6 @@
     <t>exstatus</t>
   </si>
   <si>
-    <t>Incompleted</t>
-  </si>
-  <si>
     <t>projectname</t>
   </si>
   <si>
@@ -495,17 +495,29 @@
   <si>
     <t>TR-11</t>
   </si>
+  <si>
+    <t>relese</t>
+  </si>
+  <si>
+    <t>testrun</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -515,34 +527,17 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="8.1999999999999993"/>
-      <color rgb="FF667084"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
@@ -551,13 +546,163 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="8.2"/>
+      <color rgb="FF667084"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <charset val="134"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -570,8 +715,194 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -579,11 +910,253 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -591,34 +1164,73 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -667,7 +1279,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="020F0302020204030204"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -700,26 +1312,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -752,23 +1347,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -930,21 +1508,16 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="22.5703125" customWidth="1"/>
+    <col min="1" max="1" width="22.575" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
   </cols>
   <sheetData>
@@ -966,18 +1539,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CF5A029-64A1-403A-837B-C32E1E2D6417}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="32.140625" customWidth="1"/>
-    <col min="2" max="2" width="19.28515625" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" customWidth="1"/>
-    <col min="4" max="4" width="14.28515625" customWidth="1"/>
+    <col min="1" max="1" width="32.1333333333333" customWidth="1"/>
+    <col min="2" max="2" width="19.2833333333333" customWidth="1"/>
+    <col min="3" max="3" width="16.425" customWidth="1"/>
+    <col min="4" max="4" width="14.2833333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1010,13 +1585,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82C5533E-46B7-404F-B141-BA8D149ED6E2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
@@ -1048,19 +1625,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67D36684-4EDA-4FF0-85DD-1EA9CD94F353}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="38.85546875" customWidth="1"/>
-    <col min="2" max="2" width="36.85546875" customWidth="1"/>
+    <col min="1" max="1" width="38.8583333333333" customWidth="1"/>
+    <col min="2" max="2" width="36.8583333333333" customWidth="1"/>
     <col min="3" max="3" width="31" customWidth="1"/>
-    <col min="4" max="4" width="28.5703125" customWidth="1"/>
-    <col min="5" max="5" width="19.140625" customWidth="1"/>
+    <col min="4" max="4" width="28.575" customWidth="1"/>
+    <col min="5" max="5" width="19.1333333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -1099,147 +1678,157 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE4B7E90-5E45-412C-A63B-679C413C3D5C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="9" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="9" t="s">
         <v>47</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51CCB92C-EDEC-48CF-89CB-C9462950544E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="9" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="9" t="s">
         <v>47</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA114ADC-2537-4EF7-8F50-85932949F6E5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="9" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="9" t="s">
         <v>47</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{042B7EE0-F346-47F6-9722-542962CA49F2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="9" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="9" t="s">
         <v>47</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988F8CE0-D2B6-4607-9F68-E84B3BB17A0A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
@@ -1271,13 +1860,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DF7D1D6-42F9-4EC1-BFA9-B2A7D34CCAC2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
@@ -1309,13 +1900,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D4354BF-6006-4215-AA04-8EA9BBA3CDF1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="27.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="27.1333333333333" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="4"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
@@ -1335,16 +1928,16 @@
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="8" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="8" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="1" t="s">
@@ -1353,13 +1946,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82C2809E-16FE-43EA-BC05-80D276E43A65}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
@@ -1379,13 +1974,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F957C3CC-73B2-4386-9703-3136A7AE8A62}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="14.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="14.8583333333333" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
@@ -1402,31 +1999,33 @@
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="8" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="C2" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="8" t="s">
         <v>18</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33EC2AFD-EEAB-4A46-AE51-DB66407041B8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="38.7109375" customWidth="1"/>
-    <col min="2" max="2" width="17.85546875" customWidth="1"/>
+    <col min="1" max="1" width="38.7083333333333" customWidth="1"/>
+    <col min="2" max="2" width="17.8583333333333" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1442,10 +2041,10 @@
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="1" t="s">
@@ -1454,18 +2053,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A085FA3-2BB3-4D74-980D-561D1731E50F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="28.42578125" customWidth="1"/>
-    <col min="2" max="2" width="31.28515625" customWidth="1"/>
+    <col min="1" max="1" width="28.425" customWidth="1"/>
+    <col min="2" max="2" width="31.2833333333333" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="28.5703125" customWidth="1"/>
+    <col min="4" max="4" width="28.575" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -1482,7 +2083,7 @@
         <v>13</v>
       </c>
       <c r="E1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1504,20 +2105,86 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{529C7ADA-95D5-4FFD-8278-7A1FFD92FC6F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="26.5703125" customWidth="1"/>
-    <col min="7" max="7" width="32.5703125" customWidth="1"/>
-    <col min="8" max="8" width="29.7109375" customWidth="1"/>
+    <col min="1" max="1" width="26.575" customWidth="1"/>
+    <col min="7" max="7" width="32.575" customWidth="1"/>
+    <col min="8" max="8" width="29.7083333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
+      <c r="A1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G2" s="5">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="7"/>
+  <sheetData>
+    <row r="1" ht="14.5" spans="1:8">
       <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
@@ -1531,19 +2198,19 @@
         <v>13</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>6</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" ht="14.5" spans="1:8">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -1560,146 +2227,88 @@
         <v>25</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G2" s="4">
         <v>1</v>
       </c>
       <c r="H2" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="6"/>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC0268C7-979F-44DB-BB29-34F2B8A2CC61}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="6">
-        <v>1</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0EDD7F5-B476-4FD1-BEDA-E531A4CC894D}">
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+      <c r="G2" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53291E11-0F73-43B9-A291-8813C6E50618}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="5"/>
   <cols>
-    <col min="2" max="2" width="18.42578125" customWidth="1"/>
-    <col min="3" max="3" width="20.42578125" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" customWidth="1"/>
+    <col min="2" max="2" width="18.425" customWidth="1"/>
+    <col min="3" max="3" width="20.425" customWidth="1"/>
+    <col min="4" max="4" width="18.425" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1720,7 +2329,7 @@
         <v>14</v>
       </c>
       <c r="F1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -1739,19 +2348,21 @@
       <c r="E2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="7" t="s">
         <v>52</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8956054-5465-4015-AEAB-67BB9851B24F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="18.28515625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="18.2833333333333" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="4"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
@@ -1789,17 +2400,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C5EDEDE-C2C9-4A01-9CD5-CB8C86EBBE08}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" customWidth="1"/>
-    <col min="2" max="2" width="33.140625" customWidth="1"/>
-    <col min="3" max="3" width="31.28515625" customWidth="1"/>
+    <col min="1" max="1" width="19.2833333333333" customWidth="1"/>
+    <col min="2" max="2" width="33.1333333333333" customWidth="1"/>
+    <col min="3" max="3" width="31.2833333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1820,10 +2433,10 @@
       <c r="A2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -1832,54 +2445,58 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20AD7FB8-5DA1-4488-9DE3-A42870B02C3F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="1" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="1" t="s">
         <v>42</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAE3D50E-9B7C-4048-BF74-2691F8F3F3B0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
-    <col min="2" max="2" width="19.85546875" customWidth="1"/>
+    <col min="2" max="2" width="19.8583333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1897,10 +2514,10 @@
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="1" t="s">
@@ -1912,17 +2529,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90FECA65-C9A0-48C7-B3DC-F9FDF05C4662}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="36.5703125" customWidth="1"/>
+    <col min="1" max="1" width="36.575" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" customWidth="1"/>
+    <col min="3" max="3" width="14.575" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1941,28 +2560,30 @@
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>49</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+        <v>62</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB0829FE-96F7-43C0-8C41-619F29B6B47C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="14" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="14" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="5"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
@@ -1975,100 +2596,46 @@
         <v>5</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>49</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60A730C5-C7A1-4920-B9BC-7469CD655A62}">
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultColWidth="17.140625" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F1" t="s">
-        <v>63</v>
-      </c>
-      <c r="G1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F2" t="s">
-        <v>66</v>
-      </c>
-      <c r="G2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C9A404D-916D-4310-B74F-6006281B7179}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="23.5703125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="23.575" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -2094,13 +2661,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C499954-818C-4267-A95A-C13609BD2025}">
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="5"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
@@ -2119,7 +2688,7 @@
         <v>14</v>
       </c>
       <c r="F1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -2138,238 +2707,299 @@
       <c r="E2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="7" t="s">
         <v>52</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
+  <cols>
+    <col min="1" max="1" width="28.425" customWidth="1"/>
+    <col min="2" max="2" width="18.1333333333333" customWidth="1"/>
+    <col min="3" max="3" width="18.425" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1184356D-1AE6-4E98-8694-D387B6BCDC24}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="28.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.140625" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+    <col min="7" max="7" width="31.425" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:8">
+      <c r="A1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="5">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
+  <cols>
+    <col min="1" max="1" width="27.7083333333333" customWidth="1"/>
+    <col min="2" max="2" width="19.425" customWidth="1"/>
+    <col min="3" max="3" width="21.1333333333333" customWidth="1"/>
+    <col min="4" max="4" width="17.425" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="3" t="s">
+      <c r="C1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{602CC745-32D4-47CB-82A6-B4E20CF5EEBB}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="3" t="s">
+      <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="5"/>
+  <cols>
+    <col min="5" max="5" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B5AA7B5-E8E5-4566-8F96-53EECD2B45C9}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50EB1A7D-DC52-4713-ABC3-596E81595BB1}">
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+      <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="5"/>
   <cols>
-    <col min="8" max="8" width="31.42578125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="I1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
-      <c r="A2" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="9">
-        <v>1</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDB454D5-570E-40AD-BB2C-FF13FAD6F69C}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="27.7109375" customWidth="1"/>
-    <col min="2" max="2" width="19.42578125" customWidth="1"/>
-    <col min="3" max="3" width="21.140625" customWidth="1"/>
-    <col min="4" max="4" width="17.42578125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>42</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{807E892B-8929-4105-B8A9-12065D70D1F4}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="12.28515625" customWidth="1"/>
-    <col min="2" max="2" width="33.42578125" customWidth="1"/>
+    <col min="1" max="1" width="12.2833333333333" customWidth="1"/>
+    <col min="2" max="2" width="33.425" customWidth="1"/>
     <col min="6" max="6" width="28" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2394,127 +3024,81 @@
       </c>
     </row>
     <row r="2" spans="1:6">
+      <c r="A2" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
+  <cols>
+    <col min="1" max="1" width="28.575" customWidth="1"/>
+    <col min="2" max="2" width="16.7083333333333" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F2" s="10" t="s">
-        <v>20</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1ED00A0B-CD51-4A4F-8051-1ED251D3C5B6}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>56</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE51A2BC-36BD-4EBA-8604-26295ECE93E9}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="28.5703125" customWidth="1"/>
-    <col min="2" max="2" width="16.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B69D1B4E-F873-4DB0-B2EA-24B046130852}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
-    <col min="2" max="2" width="15.85546875" customWidth="1"/>
-    <col min="3" max="3" width="15.28515625" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" customWidth="1"/>
-    <col min="5" max="5" width="27.140625" customWidth="1"/>
+    <col min="2" max="2" width="15.8583333333333" customWidth="1"/>
+    <col min="3" max="3" width="15.2833333333333" customWidth="1"/>
+    <col min="4" max="4" width="11.425" customWidth="1"/>
+    <col min="5" max="5" width="27.1333333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
@@ -2528,10 +3112,10 @@
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C2" t="s">
@@ -2546,18 +3130,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6166FFA-72F8-495E-9A03-1D63C7A066F4}">
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12.425" customWidth="1"/>
+    <col min="3" max="3" width="12.2833333333333" customWidth="1"/>
+    <col min="4" max="4" width="12.575" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -2581,7 +3167,7 @@
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
@@ -2602,13 +3188,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{626481C8-CDB8-4E7E-84A8-4409E5CFD495}">
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="24.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="24.1333333333333" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="5"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
@@ -2631,7 +3219,7 @@
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
@@ -2652,121 +3240,199 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="7"/>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4983F34-AE5D-40C9-BB36-540F7984E580}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="4"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="7"/>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>81</v>
+      <c r="E1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>85</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{631D63AD-491D-498E-BAC2-4C00217678C8}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+      <c r="F2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G2" s="5">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4D278FD-C072-43D7-9D65-282A374E276D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:8">
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="7"/>
+  <cols>
+    <col min="1" max="1" width="29.8583333333333" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="26.8583333333333" customWidth="1"/>
+    <col min="4" max="5" width="22.7083333333333" customWidth="1"/>
+    <col min="6" max="6" width="18.7083333333333" customWidth="1"/>
+    <col min="8" max="8" width="42.8583333333333" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="14.5" spans="1:8">
       <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
@@ -2780,19 +3446,19 @@
         <v>13</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>6</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" ht="14.5" spans="1:8">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -2809,156 +3475,142 @@
         <v>25</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G2" s="4">
         <v>1</v>
       </c>
       <c r="H2" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="7"/>
+  <sheetData>
+    <row r="1" ht="14.5" spans="1:8">
+      <c r="A1" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" ht="14.5" spans="1:8">
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>57</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{262279DB-08EA-408F-8B51-34383F1C571D}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="29.85546875" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="26.85546875" customWidth="1"/>
-    <col min="4" max="5" width="22.7109375" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="8" max="8" width="42.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" s="5" t="s">
+      <c r="G2" s="4">
+        <v>1</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="5"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="5" t="s">
+      <c r="E1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H1" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="5" t="s">
+      <c r="F1" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="6">
-        <v>1</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A5094B1-F969-40E8-B638-30CC9EEEC009}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="6">
-        <v>1</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+      <c r="F2" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1227A506-805A-4764-8A9B-E0A3E88E40BF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="26.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="26.425" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="4"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
@@ -2996,179 +3648,135 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A469181C-01B9-4C34-A427-3D7B86980067}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="8" t="s">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultColWidth="25.1333333333333" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="4"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="8" t="s">
+      <c r="E1" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="8" t="s">
-        <v>88</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F814BA2-835C-42C7-BBDB-409A7725E7FE}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="25.140625" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="8" t="s">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="7"/>
+  <cols>
+    <col min="1" max="1" width="37.8583333333333" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="8" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="8" t="s">
+      <c r="E1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+      <c r="F2" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3ACD041-5E11-4FA0-B069-3C5CC2C19A0C}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="37.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>92</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD8F4123-7EDA-4FD6-8DA8-8DB314949234}">
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="60.140625" customWidth="1"/>
-    <col min="2" max="2" width="57.42578125" customWidth="1"/>
-    <col min="3" max="3" width="51.42578125" customWidth="1"/>
+    <col min="1" max="1" width="60.1333333333333" customWidth="1"/>
+    <col min="2" max="2" width="57.425" customWidth="1"/>
+    <col min="3" max="3" width="51.425" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="22.5703125" customWidth="1"/>
-    <col min="6" max="6" width="11.85546875" customWidth="1"/>
+    <col min="5" max="5" width="22.575" customWidth="1"/>
+    <col min="6" max="6" width="11.8583333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -3219,21 +3827,23 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C530097-25F5-490E-B95D-3F7CE84A8B5A}">
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="35.28515625" customWidth="1"/>
-    <col min="2" max="2" width="39.7109375" customWidth="1"/>
-    <col min="3" max="3" width="37.5703125" customWidth="1"/>
-    <col min="4" max="4" width="24.42578125" customWidth="1"/>
-    <col min="5" max="5" width="14.42578125" customWidth="1"/>
+    <col min="1" max="1" width="35.2833333333333" customWidth="1"/>
+    <col min="2" max="2" width="39.7083333333333" customWidth="1"/>
+    <col min="3" max="3" width="37.575" customWidth="1"/>
+    <col min="4" max="4" width="24.425" customWidth="1"/>
+    <col min="5" max="5" width="14.425" customWidth="1"/>
     <col min="6" max="6" width="17" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" customWidth="1"/>
+    <col min="7" max="7" width="14.425" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -3285,18 +3895,20 @@
         <v>85</v>
       </c>
       <c r="H2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9928D07B-EC4B-4FB7-A544-ACD154E60B5A}">
+        <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="7"/>
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
@@ -3352,13 +3964,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65567DB9-F4A5-4991-BBBB-B0966631BE02}">
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="7"/>
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
@@ -3409,18 +4023,20 @@
         <v>85</v>
       </c>
       <c r="H2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABC46D15-7486-489E-8CFB-3757E997A7F3}">
+        <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -3446,13 +4062,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3493DC4-C417-4C28-8EE7-B8304F691C93}">
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -3478,13 +4096,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5737D2A7-9183-4F17-A1A0-D46634DAE493}">
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -3510,17 +4130,53 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE4FC528-53EE-4A96-BCAB-C9D74542958B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="22.85546875" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" customWidth="1"/>
-    <col min="3" max="3" width="20.5703125" customWidth="1"/>
+    <col min="1" max="1" width="22.8583333333333" customWidth="1"/>
+    <col min="2" max="2" width="17.7083333333333" customWidth="1"/>
+    <col min="3" max="3" width="20.575" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3547,45 +4203,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB8F0DCE-952C-484A-B429-28D41548BB7A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8840A44C-6BDB-471E-B7F3-2A372A7C4B5B}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="19.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="19.425" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -3611,13 +4237,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B9B72EB-97C0-4405-94F5-046368E85D80}">
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -3643,13 +4271,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09FCDA05-EF6F-42AB-9CB8-2EAB3573710B}">
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
@@ -3681,13 +4311,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B038332-BB0C-4E20-A6A2-9F7526C4D248}">
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
@@ -3719,13 +4351,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E093CE88-AC07-4898-81D8-6061F00C4D92}">
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="4"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
@@ -3763,13 +4397,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAFE400E-814A-476C-9FF3-1A384DD6A39D}">
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="6"/>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
@@ -3811,7 +4447,7 @@
         <v>125</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>9</v>
@@ -3819,13 +4455,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DBB2522-C0DE-4085-ADBF-7FE9C84B6F31}">
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="18.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="18.1333333333333" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
@@ -3857,13 +4495,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E1B32B0-F3F2-47B6-A128-2992201FC613}">
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="19.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="19.7083333333333" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -3889,13 +4529,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E7BB830-EB99-49CB-BF04-A0C705F8DA3E}">
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -3921,18 +4563,54 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E32429F3-AABC-45DD-B647-116877616A3B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" customWidth="1"/>
+    <col min="1" max="1" width="19.8583333333333" customWidth="1"/>
+    <col min="2" max="2" width="15.7083333333333" customWidth="1"/>
+    <col min="3" max="3" width="18.7083333333333" customWidth="1"/>
+    <col min="4" max="4" width="17.575" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -3971,45 +4649,49 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57E304D9-C2CF-4191-B2D5-F19B4BAEF075}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>107</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>126</v>
+        <v>108</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>127</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+        <v>112</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D109D0F-DF6D-4E54-A85C-F205345D7EE8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -4035,13 +4717,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58DC1A5D-B5FD-4AF6-9CE0-84600C30705B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -4067,13 +4751,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AF5112D-7B38-4AF6-8BE8-212DFAB6FA1F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -4099,45 +4785,179 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C3DEA2D-3BC8-46BF-82C0-FA72EAFC6314}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="8.725" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="8.66666666666667" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultColWidth="8.725" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="5"/>
+  <sheetData>
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>107</v>
+        <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>108</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
+        <v>5</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>110</v>
+        <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>111</v>
+        <v>7</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>112</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+        <v>49</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="8.725" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="8.725" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84A7507B-FC99-4CF2-AE3D-BE5F23D6F22B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultColWidth="22.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="22.8583333333333" defaultRowHeight="14" outlineLevelRow="1"/>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
@@ -4145,23 +4965,25 @@
       </c>
     </row>
     <row r="2" spans="1:1">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="8" t="s">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{080476E3-62E4-4BCA-8888-D4B5BD88468D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="28.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.5703125" customWidth="1"/>
-    <col min="3" max="3" width="20.7109375" customWidth="1"/>
+    <col min="1" max="1" width="28.7083333333333" customWidth="1"/>
+    <col min="2" max="2" width="23.575" customWidth="1"/>
+    <col min="3" max="3" width="20.7083333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4188,5 +5010,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>